<commit_message>
feat: implemented v2 braking physics rework
Coordinated changes across tyres.ini, electronics.ini, abs_control.lut
and aero.ini to address unrealistic braking behaviour identified in
baseline telemetry analysis.
</commit_message>
<xml_diff>
--- a/analysis/gt3_braking_telemetry_analysis.xlsx
+++ b/analysis/gt3_braking_telemetry_analysis.xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tautv\Desktop\SimuPilot\analysis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BCAC54EB-4F05-4BC4-97ED-EC05F4458884}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E4823FE8-BBE3-46B6-9605-BCDF571E61D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21840" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21840" tabRatio="500" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Test Comparison" sheetId="1" r:id="rId1"/>
     <sheet name="Braking Zone Analysis" sheetId="5" r:id="rId2"/>
     <sheet name="Key Findings" sheetId="3" r:id="rId3"/>
-    <sheet name="Proposed Physics Modifications" sheetId="4" r:id="rId4"/>
+    <sheet name="Proposed Physics Changes" sheetId="6" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029" iterateDelta="1E-4"/>
   <extLst>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="140" uniqueCount="120">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="176" uniqueCount="142">
   <si>
     <t>Metric</t>
   </si>
@@ -176,114 +176,18 @@
     <t>Parameter</t>
   </si>
   <si>
-    <t>Current Value</t>
-  </si>
-  <si>
-    <t>Suggested Value</t>
-  </si>
-  <si>
     <t>Rationale</t>
   </si>
   <si>
     <t>tyres.ini</t>
   </si>
   <si>
-    <t>DX_REF</t>
-  </si>
-  <si>
-    <t>0.20</t>
-  </si>
-  <si>
-    <t>0.13–0.15</t>
-  </si>
-  <si>
-    <t>Reduces sustained peak grip — addresses Finding 1 (no G decay)</t>
-  </si>
-  <si>
-    <t>FALLOFF_SPEED</t>
-  </si>
-  <si>
     <t>1.0</t>
   </si>
   <si>
-    <t>1.2–1.5</t>
-  </si>
-  <si>
-    <t>Faster grip falloff with slip speed — reinforces G decay</t>
-  </si>
-  <si>
-    <t>COMBINED_FACTOR</t>
-  </si>
-  <si>
-    <t>0.95</t>
-  </si>
-  <si>
-    <t>0.82</t>
-  </si>
-  <si>
-    <t>Stronger combined slip penalty — addresses Finding 2 (friction circle)</t>
-  </si>
-  <si>
-    <t>DX0</t>
-  </si>
-  <si>
-    <t>1.72</t>
-  </si>
-  <si>
-    <t>1.65</t>
-  </si>
-  <si>
-    <t>Lower peak longitudinal friction coefficient</t>
-  </si>
-  <si>
-    <t>DX1</t>
-  </si>
-  <si>
-    <t>1.82</t>
-  </si>
-  <si>
-    <t>1.75</t>
-  </si>
-  <si>
-    <t>Lower sliding longitudinal friction coefficient</t>
-  </si>
-  <si>
-    <t>LS_EXP</t>
-  </si>
-  <si>
-    <t>0.55</t>
-  </si>
-  <si>
-    <t>0.65–0.75</t>
-  </si>
-  <si>
-    <t>Sharper load sensitivity — more penalty for overloading tyre</t>
-  </si>
-  <si>
-    <t>ctrl.ini</t>
-  </si>
-  <si>
-    <t>ABS threshold</t>
-  </si>
-  <si>
-    <t>Review</t>
-  </si>
-  <si>
-    <t>Tighten ABS intervention window — addresses Finding 3 (ABS too forgiving)</t>
-  </si>
-  <si>
     <t>aero.ini</t>
   </si>
   <si>
-    <t>Front wing pitch coeff</t>
-  </si>
-  <si>
-    <t>+~20%</t>
-  </si>
-  <si>
-    <t>Increased front downforce for more realistic braking stability</t>
-  </si>
-  <si>
     <t xml:space="preserve"> Friction Circle Not Enforced — Combined Slip Penalty Too Weak</t>
   </si>
   <si>
@@ -308,9 +212,6 @@
     <t>Test B (threshold modulation + proper trail brake) is 0.829s per lap slower than Test A (sustained 100% brake). The three behaviours above compound to actively penalise correct driving - maximum slam-and-hold is the fastest approach in the unmodified AC tyre model.</t>
   </si>
   <si>
-    <t>Proposed Physics Modifications — Addressing Identified Behaviours</t>
-  </si>
-  <si>
     <t>Key Findings - Unmodified AC GT3 Braking Physics</t>
   </si>
   <si>
@@ -399,6 +300,173 @@
   </si>
   <si>
     <t>Entry speed (kmph)</t>
+  </si>
+  <si>
+    <t>20% increase to front wing lift coefficient multiplier. Increases front downforce to improve braking stability and weight transfer. Note: ANGLE=2 is already at peak CL per wing_front_AOA_CL.lut — angle left unchanged.</t>
+  </si>
+  <si>
+    <t>1.2</t>
+  </si>
+  <si>
+    <t>CL_GAIN (WING_1 front)</t>
+  </si>
+  <si>
+    <t>Upper ceiling of ABS tolerance reduced. Prevents extreme over-drive at any ABS setting.</t>
+  </si>
+  <si>
+    <t>0.15</t>
+  </si>
+  <si>
+    <t>0.17</t>
+  </si>
+  <si>
+    <t>Level 11 target
+(maximum)</t>
+  </si>
+  <si>
+    <t>abs_control.lut</t>
+  </si>
+  <si>
+    <t>At the default test ABS level (7), intervention threshold drops from 13% to 11%. Directly comparable to measured peak slip FL of −14.50% in Test A baseline — ABS will now manage slip more tightly.</t>
+  </si>
+  <si>
+    <t>0.11</t>
+  </si>
+  <si>
+    <t>0.13</t>
+  </si>
+  <si>
+    <t>Level 7 target
+(test default)</t>
+  </si>
+  <si>
+    <t>Entire ABS intervention curve shifted down by 0.02 at every level. Maximum slip at level 11 reduced from 17% to 15%. ABS intervenes earlier — over-driving the ABS now produces a measurable efficiency penalty. Addresses Finding 3.</t>
+  </si>
+  <si>
+    <t>0.04</t>
+  </si>
+  <si>
+    <t>0.06</t>
+  </si>
+  <si>
+    <t>Level 0 target</t>
+  </si>
+  <si>
+    <t>Tightens ABS reference slip target from 12% to 9%. Closer to optimal braking slip window identified in telemetry. Addresses Finding 3.</t>
+  </si>
+  <si>
+    <t>0.09</t>
+  </si>
+  <si>
+    <t>0.12</t>
+  </si>
+  <si>
+    <t>SLIP_RATIO_LIMIT</t>
+  </si>
+  <si>
+    <t>electronics.ini</t>
+  </si>
+  <si>
+    <t>Removes 10% longitudinal stiffness bonus. Reduces the independent longitudinal force generation that undermines combined slip penalty. Addresses Finding 2.</t>
+  </si>
+  <si>
+    <t>1.1</t>
+  </si>
+  <si>
+    <t>CX_MULT (all)</t>
+  </si>
+  <si>
+    <t>Reduces the bonus longitudinal friction applied specifically during braking. Weakens longitudinal dominance, helping friction circle enforcement. Addresses Findings 2 and 3.</t>
+  </si>
+  <si>
+    <t>BRAKE_DX_MOD (all)</t>
+  </si>
+  <si>
+    <t>Same increase applied to rear. Rear kept slightly higher than front to maintain balance.</t>
+  </si>
+  <si>
+    <t>0.88</t>
+  </si>
+  <si>
+    <t>0.8144</t>
+  </si>
+  <si>
+    <t>LS_EXPX (Rear, all)</t>
+  </si>
+  <si>
+    <t>Increases longitudinal load sensitivity — tyre is more responsive to load changes during braking. Reinforces G decay (Finding 1).</t>
+  </si>
+  <si>
+    <t>0.87</t>
+  </si>
+  <si>
+    <t>0.8017</t>
+  </si>
+  <si>
+    <t>LS_EXPX (Front, all)</t>
+  </si>
+  <si>
+    <t>Same DX &lt; DY differential applied to hard compound.</t>
+  </si>
+  <si>
+    <t>1.52</t>
+  </si>
+  <si>
+    <t>1.54</t>
+  </si>
+  <si>
+    <t>DY_REF (Hard F/R)</t>
+  </si>
+  <si>
+    <t>Same DX &lt; DY differential applied to medium compound.</t>
+  </si>
+  <si>
+    <t>1.56</t>
+  </si>
+  <si>
+    <t>DY_REF (Medium F/R)</t>
+  </si>
+  <si>
+    <t>Reduced less than DX_REF to create DX &lt; DY ratio — begins enforcing a friction ellipse rather than a circle. Addresses Finding 2.</t>
+  </si>
+  <si>
+    <t>1.58</t>
+  </si>
+  <si>
+    <t>DY_REF (Soft F/R)</t>
+  </si>
+  <si>
+    <t>Same reduction applied to hard compound. Compound hierarchy preserved.</t>
+  </si>
+  <si>
+    <t>1.50</t>
+  </si>
+  <si>
+    <t>DX_REF (Hard F/R)</t>
+  </si>
+  <si>
+    <t>Same reduction applied to medium compound. Compound hierarchy preserved (−0.04 step maintained across soft/medium/hard).</t>
+  </si>
+  <si>
+    <t>DX_REF (Medium F/R)</t>
+  </si>
+  <si>
+    <t>Reduces peak longitudinal friction reference. Addresses Finding 1 — lowers sustained decel ceiling so grip falls off more naturally.</t>
+  </si>
+  <si>
+    <t>DX_REF (Soft F/R)</t>
+  </si>
+  <si>
+    <t>v2 Value</t>
+  </si>
+  <si>
+    <t>Stock Value</t>
+  </si>
+  <si>
+    <t xml:space="preserve">                                       All changes applied to v2_braking_rework_1 · Addresses Findings 1, 2, 3 · Medium tyre is primary test compound</t>
+  </si>
+  <si>
+    <t>Physics Modifications — v2 Implemented Changes</t>
   </si>
 </sst>
 </file>
@@ -571,101 +639,101 @@
   </cellStyleXfs>
   <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="6" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="6" fillId="10" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="11" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="6" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="6" fillId="10" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -939,410 +1007,410 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="6" t="s">
-        <v>92</v>
-      </c>
-      <c r="B1" s="6"/>
-      <c r="C1" s="6"/>
-      <c r="D1" s="6"/>
+      <c r="A1" s="28" t="s">
+        <v>59</v>
+      </c>
+      <c r="B1" s="28"/>
+      <c r="C1" s="28"/>
+      <c r="D1" s="28"/>
     </row>
     <row r="2" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="5" t="s">
-        <v>91</v>
-      </c>
-      <c r="B2" s="5"/>
-      <c r="C2" s="5"/>
-      <c r="D2" s="5"/>
+      <c r="A2" s="29" t="s">
+        <v>58</v>
+      </c>
+      <c r="B2" s="29"/>
+      <c r="C2" s="29"/>
+      <c r="D2" s="29"/>
     </row>
     <row r="3" spans="1:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="7" t="s">
+      <c r="A3" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="8" t="s">
+      <c r="B3" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="9" t="s">
+      <c r="C3" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D3" s="10" t="s">
+      <c r="D3" s="4" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="4" t="s">
+      <c r="A4" s="27" t="s">
         <v>4</v>
       </c>
-      <c r="B4" s="4"/>
-      <c r="C4" s="4"/>
-      <c r="D4" s="4"/>
+      <c r="B4" s="27"/>
+      <c r="C4" s="27"/>
+      <c r="D4" s="27"/>
     </row>
     <row r="5" spans="1:4" ht="43.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="11" t="s">
+      <c r="A5" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="B5" s="12" t="s">
+      <c r="B5" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="C5" s="12" t="s">
+      <c r="C5" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="D5" s="12" t="s">
+      <c r="D5" s="6" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="4" t="s">
+      <c r="A6" s="27" t="s">
         <v>9</v>
       </c>
-      <c r="B6" s="4"/>
-      <c r="C6" s="4"/>
-      <c r="D6" s="4"/>
+      <c r="B6" s="27"/>
+      <c r="C6" s="27"/>
+      <c r="D6" s="27"/>
     </row>
     <row r="7" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="11" t="s">
-        <v>119</v>
-      </c>
-      <c r="B7" s="12">
+      <c r="A7" s="5" t="s">
+        <v>86</v>
+      </c>
+      <c r="B7" s="6">
         <v>273.60000000000002</v>
       </c>
-      <c r="C7" s="12">
+      <c r="C7" s="6">
         <v>271.8</v>
       </c>
-      <c r="D7" s="12">
+      <c r="D7" s="6">
         <v>272.60000000000002</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="4" t="s">
+      <c r="A8" s="27" t="s">
         <v>10</v>
       </c>
-      <c r="B8" s="4"/>
-      <c r="C8" s="4"/>
-      <c r="D8" s="4"/>
+      <c r="B8" s="27"/>
+      <c r="C8" s="27"/>
+      <c r="D8" s="27"/>
     </row>
     <row r="9" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="11" t="s">
+      <c r="A9" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="B9" s="12">
+      <c r="B9" s="6">
         <v>-2.2753000000000001</v>
       </c>
-      <c r="C9" s="12">
+      <c r="C9" s="6">
         <v>-1.9602999999999999</v>
       </c>
-      <c r="D9" s="12">
+      <c r="D9" s="6">
         <v>-2.0811999999999999</v>
       </c>
     </row>
     <row r="10" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="11" t="s">
-        <v>101</v>
-      </c>
-      <c r="B10" s="13">
+      <c r="A10" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="B10" s="7">
         <v>-1.6395</v>
       </c>
-      <c r="C10" s="13">
+      <c r="C10" s="7">
         <v>-1.2253000000000001</v>
       </c>
-      <c r="D10" s="13">
+      <c r="D10" s="7">
         <v>-1.5885</v>
       </c>
     </row>
     <row r="11" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="11" t="s">
+      <c r="A11" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="B11" s="12">
+      <c r="B11" s="6">
         <v>-1.5952</v>
       </c>
-      <c r="C11" s="12">
+      <c r="C11" s="6">
         <v>-1.1148</v>
       </c>
-      <c r="D11" s="12">
+      <c r="D11" s="6">
         <v>-1.1608000000000001</v>
       </c>
     </row>
     <row r="12" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="11" t="s">
+      <c r="A12" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="B12" s="13" t="s">
+      <c r="B12" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="C12" s="13" t="s">
+      <c r="C12" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="D12" s="13" t="s">
+      <c r="D12" s="7" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="13" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="11" t="s">
+      <c r="A13" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="B13" s="12">
+      <c r="B13" s="6">
         <v>5.1100000000000003</v>
       </c>
-      <c r="C13" s="12">
+      <c r="C13" s="6">
         <v>6.43</v>
       </c>
-      <c r="D13" s="12">
+      <c r="D13" s="6">
         <v>7.25</v>
       </c>
     </row>
     <row r="14" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="11" t="s">
-        <v>98</v>
-      </c>
-      <c r="B14" s="13">
+      <c r="A14" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="B14" s="7">
         <v>-2.2753000000000001</v>
       </c>
-      <c r="C14" s="13" t="s">
+      <c r="C14" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="D14" s="13">
+      <c r="D14" s="7">
         <v>-2.0811999999999999</v>
       </c>
     </row>
     <row r="15" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="11" t="s">
-        <v>99</v>
-      </c>
-      <c r="B15" s="12">
+      <c r="A15" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="B15" s="6">
         <v>-1.5969</v>
       </c>
-      <c r="C15" s="12" t="s">
+      <c r="C15" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="D15" s="12">
+      <c r="D15" s="6">
         <v>-1.5345</v>
       </c>
     </row>
     <row r="16" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="11" t="s">
-        <v>100</v>
-      </c>
-      <c r="B16" s="13">
+      <c r="A16" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="B16" s="7">
         <v>-1.8193999999999999</v>
       </c>
-      <c r="C16" s="13" t="s">
+      <c r="C16" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="D16" s="13">
+      <c r="D16" s="7">
         <v>-1.7806999999999999</v>
       </c>
     </row>
     <row r="17" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="4" t="s">
+      <c r="A17" s="27" t="s">
         <v>19</v>
       </c>
-      <c r="B17" s="4"/>
-      <c r="C17" s="4"/>
-      <c r="D17" s="4"/>
+      <c r="B17" s="27"/>
+      <c r="C17" s="27"/>
+      <c r="D17" s="27"/>
     </row>
     <row r="18" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="11" t="s">
+      <c r="A18" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="B18" s="12">
+      <c r="B18" s="6">
         <v>750</v>
       </c>
-      <c r="C18" s="12">
+      <c r="C18" s="6">
         <v>707</v>
       </c>
-      <c r="D18" s="12">
+      <c r="D18" s="6">
         <v>739</v>
       </c>
     </row>
     <row r="19" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="11" t="s">
+      <c r="A19" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="B19" s="13">
+      <c r="B19" s="7">
         <v>881</v>
       </c>
-      <c r="C19" s="13">
+      <c r="C19" s="7">
         <v>886</v>
       </c>
-      <c r="D19" s="13">
+      <c r="D19" s="7">
         <v>896</v>
       </c>
     </row>
     <row r="20" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="11" t="s">
-        <v>117</v>
-      </c>
-      <c r="B20" s="12">
+      <c r="A20" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="B20" s="6">
         <v>69</v>
       </c>
-      <c r="C20" s="12">
+      <c r="C20" s="6">
         <v>80.2</v>
       </c>
-      <c r="D20" s="12">
+      <c r="D20" s="6">
         <v>67.2</v>
       </c>
     </row>
     <row r="21" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="11" t="s">
+      <c r="A21" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="B21" s="13">
+      <c r="B21" s="7">
         <v>916</v>
       </c>
-      <c r="C21" s="13">
+      <c r="C21" s="7">
         <v>917</v>
       </c>
-      <c r="D21" s="13">
+      <c r="D21" s="7">
         <v>911</v>
       </c>
     </row>
     <row r="22" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="4" t="s">
+      <c r="A22" s="27" t="s">
         <v>23</v>
       </c>
-      <c r="B22" s="4"/>
-      <c r="C22" s="4"/>
-      <c r="D22" s="4"/>
+      <c r="B22" s="27"/>
+      <c r="C22" s="27"/>
+      <c r="D22" s="27"/>
     </row>
     <row r="23" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="11" t="s">
+      <c r="A23" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="B23" s="12" t="s">
+      <c r="B23" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="C23" s="12" t="s">
+      <c r="C23" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="D23" s="12" t="s">
+      <c r="D23" s="6" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="24" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="11" t="s">
+      <c r="A24" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="B24" s="13" t="s">
-        <v>93</v>
-      </c>
-      <c r="C24" s="13" t="s">
+      <c r="B24" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="C24" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="D24" s="13" t="s">
-        <v>94</v>
+      <c r="D24" s="7" t="s">
+        <v>61</v>
       </c>
     </row>
     <row r="25" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="4" t="s">
+      <c r="A25" s="27" t="s">
         <v>28</v>
       </c>
-      <c r="B25" s="4"/>
-      <c r="C25" s="4"/>
-      <c r="D25" s="4"/>
+      <c r="B25" s="27"/>
+      <c r="C25" s="27"/>
+      <c r="D25" s="27"/>
     </row>
     <row r="26" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="11" t="s">
+      <c r="A26" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="B26" s="12">
+      <c r="B26" s="6">
         <v>-14.5</v>
       </c>
-      <c r="C26" s="12">
+      <c r="C26" s="6">
         <v>-7.98</v>
       </c>
-      <c r="D26" s="12">
+      <c r="D26" s="6">
         <v>-12.82</v>
       </c>
     </row>
     <row r="27" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="11" t="s">
+      <c r="A27" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="B27" s="13">
+      <c r="B27" s="7">
         <v>-14.73</v>
       </c>
-      <c r="C27" s="13">
+      <c r="C27" s="7">
         <v>-10.35</v>
       </c>
-      <c r="D27" s="13">
+      <c r="D27" s="7">
         <v>-13.84</v>
       </c>
     </row>
     <row r="28" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="11" t="s">
-        <v>95</v>
-      </c>
-      <c r="B28" s="12">
+      <c r="A28" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="B28" s="6">
         <v>-9.19</v>
       </c>
-      <c r="C28" s="12" t="s">
+      <c r="C28" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="D28" s="12">
+      <c r="D28" s="6">
         <v>-9.15</v>
       </c>
     </row>
     <row r="29" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="11" t="s">
-        <v>96</v>
-      </c>
-      <c r="B29" s="13" t="s">
+      <c r="A29" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="B29" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="C29" s="13">
+      <c r="C29" s="7">
         <v>-4.2</v>
       </c>
-      <c r="D29" s="13" t="s">
+      <c r="D29" s="7" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="30" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="11" t="s">
-        <v>97</v>
-      </c>
-      <c r="B30" s="12">
+      <c r="A30" s="5" t="s">
+        <v>64</v>
+      </c>
+      <c r="B30" s="6">
         <v>-8</v>
       </c>
-      <c r="C30" s="12">
+      <c r="C30" s="6">
         <v>-2.56</v>
       </c>
-      <c r="D30" s="12" t="s">
+      <c r="D30" s="6" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="31" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="4" t="s">
+      <c r="A31" s="27" t="s">
         <v>31</v>
       </c>
-      <c r="B31" s="4"/>
-      <c r="C31" s="4"/>
-      <c r="D31" s="4"/>
+      <c r="B31" s="27"/>
+      <c r="C31" s="27"/>
+      <c r="D31" s="27"/>
     </row>
     <row r="32" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="11" t="s">
+      <c r="A32" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="B32" s="12" t="s">
+      <c r="B32" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="C32" s="12" t="s">
+      <c r="C32" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="D32" s="12" t="s">
+      <c r="D32" s="6" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="33" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="11" t="s">
+      <c r="A33" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="B33" s="13" t="s">
+      <c r="B33" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="C33" s="13" t="s">
+      <c r="C33" s="7" t="s">
         <v>37</v>
       </c>
-      <c r="D33" s="13" t="s">
+      <c r="D33" s="7" t="s">
         <v>38</v>
       </c>
     </row>
@@ -1373,224 +1441,224 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="3" t="s">
-        <v>113</v>
-      </c>
-      <c r="B1" s="3"/>
-      <c r="C1" s="3"/>
-      <c r="D1" s="3"/>
+      <c r="A1" s="30" t="s">
+        <v>80</v>
+      </c>
+      <c r="B1" s="30"/>
+      <c r="C1" s="30"/>
+      <c r="D1" s="30"/>
     </row>
     <row r="2" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="2" t="s">
-        <v>114</v>
-      </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
+      <c r="A2" s="31" t="s">
+        <v>81</v>
+      </c>
+      <c r="B2" s="31"/>
+      <c r="C2" s="31"/>
+      <c r="D2" s="31"/>
     </row>
     <row r="3" spans="1:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="7" t="s">
+      <c r="A3" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="8" t="s">
-        <v>112</v>
-      </c>
-      <c r="C3" s="9" t="s">
-        <v>111</v>
-      </c>
-      <c r="D3" s="10" t="s">
-        <v>110</v>
+      <c r="B3" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>77</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="4" t="s">
-        <v>109</v>
-      </c>
-      <c r="B4" s="4"/>
-      <c r="C4" s="4"/>
-      <c r="D4" s="4"/>
+      <c r="A4" s="27" t="s">
+        <v>76</v>
+      </c>
+      <c r="B4" s="27"/>
+      <c r="C4" s="27"/>
+      <c r="D4" s="27"/>
     </row>
     <row r="5" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="11" t="s">
+      <c r="A5" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="B5" s="31">
+      <c r="B5" s="25">
         <v>750</v>
       </c>
-      <c r="C5" s="31">
+      <c r="C5" s="25">
         <v>706</v>
       </c>
-      <c r="D5" s="31">
+      <c r="D5" s="25">
         <v>739</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="11" t="s">
-        <v>108</v>
-      </c>
-      <c r="B6" s="32">
+      <c r="A6" s="5" t="s">
+        <v>75</v>
+      </c>
+      <c r="B6" s="26">
         <v>10.5</v>
       </c>
-      <c r="C6" s="32">
+      <c r="C6" s="26">
         <v>9.9499999999999993</v>
       </c>
-      <c r="D6" s="32">
+      <c r="D6" s="26">
         <v>10.4</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="11" t="s">
-        <v>118</v>
-      </c>
-      <c r="B7" s="31">
+      <c r="A7" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="B7" s="25">
         <v>273.60000000000002</v>
       </c>
-      <c r="C7" s="31">
+      <c r="C7" s="25">
         <v>271.8</v>
       </c>
-      <c r="D7" s="31">
+      <c r="D7" s="25">
         <v>272.60000000000002</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="4" t="s">
-        <v>107</v>
-      </c>
-      <c r="B8" s="4"/>
-      <c r="C8" s="4"/>
-      <c r="D8" s="4"/>
+      <c r="A8" s="27" t="s">
+        <v>74</v>
+      </c>
+      <c r="B8" s="27"/>
+      <c r="C8" s="27"/>
+      <c r="D8" s="27"/>
     </row>
     <row r="9" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="11" t="s">
+      <c r="A9" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="B9" s="31">
+      <c r="B9" s="25">
         <v>916</v>
       </c>
-      <c r="C9" s="31">
+      <c r="C9" s="25">
         <v>914</v>
       </c>
-      <c r="D9" s="31">
+      <c r="D9" s="25">
         <v>911</v>
       </c>
     </row>
     <row r="10" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="11" t="s">
-        <v>106</v>
-      </c>
-      <c r="B10" s="32">
+      <c r="A10" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="B10" s="26">
         <v>14.2</v>
       </c>
-      <c r="C10" s="32">
+      <c r="C10" s="26">
         <v>14.55</v>
       </c>
-      <c r="D10" s="32">
+      <c r="D10" s="26">
         <v>14.35</v>
       </c>
     </row>
     <row r="11" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="11" t="s">
-        <v>117</v>
-      </c>
-      <c r="B11" s="31">
+      <c r="A11" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="B11" s="25">
         <v>69</v>
       </c>
-      <c r="C11" s="31">
+      <c r="C11" s="25">
         <v>80</v>
       </c>
-      <c r="D11" s="31">
+      <c r="D11" s="25">
         <v>67.2</v>
       </c>
     </row>
     <row r="12" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="4" t="s">
-        <v>105</v>
-      </c>
-      <c r="B12" s="4"/>
-      <c r="C12" s="4"/>
-      <c r="D12" s="4"/>
+      <c r="A12" s="27" t="s">
+        <v>72</v>
+      </c>
+      <c r="B12" s="27"/>
+      <c r="C12" s="27"/>
+      <c r="D12" s="27"/>
     </row>
     <row r="13" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="11" t="s">
-        <v>104</v>
-      </c>
-      <c r="B13" s="29">
-        <f>B9-B5</f>
+      <c r="A13" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="B13" s="23">
+        <f t="shared" ref="B13:D14" si="0">B9-B5</f>
         <v>166</v>
       </c>
-      <c r="C13" s="29">
-        <f>C9-C5</f>
+      <c r="C13" s="23">
+        <f t="shared" si="0"/>
         <v>208</v>
       </c>
-      <c r="D13" s="29">
-        <f>D9-D5</f>
+      <c r="D13" s="23">
+        <f t="shared" si="0"/>
         <v>172</v>
       </c>
     </row>
     <row r="14" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="11" t="s">
-        <v>103</v>
-      </c>
-      <c r="B14" s="30">
-        <f>B10-B6</f>
+      <c r="A14" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="B14" s="24">
+        <f t="shared" si="0"/>
         <v>3.6999999999999993</v>
       </c>
-      <c r="C14" s="30">
-        <f>C10-C6</f>
+      <c r="C14" s="24">
+        <f t="shared" si="0"/>
         <v>4.6000000000000014</v>
       </c>
-      <c r="D14" s="30">
-        <f>D10-D6</f>
+      <c r="D14" s="24">
+        <f t="shared" si="0"/>
         <v>3.9499999999999993</v>
       </c>
     </row>
     <row r="15" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="11" t="s">
-        <v>116</v>
-      </c>
-      <c r="B15" s="29">
+      <c r="A15" s="5" t="s">
+        <v>83</v>
+      </c>
+      <c r="B15" s="23">
         <f>B7-B11</f>
         <v>204.60000000000002</v>
       </c>
-      <c r="C15" s="29">
+      <c r="C15" s="23">
         <f>C7-C11</f>
         <v>191.8</v>
       </c>
-      <c r="D15" s="29">
+      <c r="D15" s="23">
         <f>D7-D11</f>
         <v>205.40000000000003</v>
       </c>
     </row>
     <row r="16" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="11" t="s">
-        <v>115</v>
-      </c>
-      <c r="B16" s="30">
+      <c r="A16" s="5" t="s">
+        <v>82</v>
+      </c>
+      <c r="B16" s="24">
         <f>(B7-B11)/( B10-B6)</f>
         <v>55.297297297297312</v>
       </c>
-      <c r="C16" s="30">
+      <c r="C16" s="24">
         <f>(C7-C11)/(C10-C6)</f>
         <v>41.695652173913032</v>
       </c>
-      <c r="D16" s="30">
+      <c r="D16" s="24">
         <f>(D7-D11)/(D10-D6)</f>
         <v>52.000000000000021</v>
       </c>
     </row>
     <row r="17" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="11" t="s">
-        <v>102</v>
-      </c>
-      <c r="B17" s="29">
+      <c r="A17" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="B17" s="23">
         <f>(B7-B11)/3.6/(B10-B6)</f>
         <v>15.360360360360364</v>
       </c>
-      <c r="C17" s="29">
+      <c r="C17" s="23">
         <f>(C7-C11)/3.6/(C10-C6)</f>
         <v>11.58212560386473</v>
       </c>
-      <c r="D17" s="29">
+      <c r="D17" s="23">
         <f>(D7-D11)/3.6/(D10-D6)</f>
         <v>14.44444444444445</v>
       </c>
@@ -1618,66 +1686,66 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="3" t="s">
-        <v>90</v>
-      </c>
-      <c r="B1" s="3"/>
+      <c r="A1" s="30" t="s">
+        <v>57</v>
+      </c>
+      <c r="B1" s="30"/>
     </row>
     <row r="2" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="15" t="s">
+      <c r="A2" s="9" t="s">
         <v>39</v>
       </c>
-      <c r="B2" s="16" t="s">
-        <v>82</v>
+      <c r="B2" s="10" t="s">
+        <v>50</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="49.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
-        <v>86</v>
-      </c>
-      <c r="B3" s="1"/>
+      <c r="A3" s="32" t="s">
+        <v>54</v>
+      </c>
+      <c r="B3" s="32"/>
     </row>
     <row r="4" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="17" t="s">
+      <c r="A4" s="11" t="s">
         <v>40</v>
       </c>
-      <c r="B4" s="18" t="s">
-        <v>81</v>
+      <c r="B4" s="12" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="41.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="1" t="s">
-        <v>87</v>
-      </c>
-      <c r="B5" s="1"/>
+      <c r="A5" s="32" t="s">
+        <v>55</v>
+      </c>
+      <c r="B5" s="32"/>
     </row>
     <row r="6" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="19" t="s">
+      <c r="A6" s="13" t="s">
         <v>41</v>
       </c>
-      <c r="B6" s="20" t="s">
-        <v>83</v>
+      <c r="B6" s="14" t="s">
+        <v>51</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="40.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="1" t="s">
-        <v>85</v>
-      </c>
-      <c r="B7" s="1"/>
+      <c r="A7" s="32" t="s">
+        <v>53</v>
+      </c>
+      <c r="B7" s="32"/>
     </row>
     <row r="8" spans="1:2" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="21" t="s">
+      <c r="A8" s="15" t="s">
         <v>42</v>
       </c>
-      <c r="B8" s="22" t="s">
-        <v>84</v>
+      <c r="B8" s="16" t="s">
+        <v>52</v>
       </c>
     </row>
     <row r="9" spans="1:2" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="1" t="s">
-        <v>88</v>
-      </c>
-      <c r="B9" s="1"/>
+      <c r="A9" s="32" t="s">
+        <v>56</v>
+      </c>
+      <c r="B9" s="32"/>
     </row>
     <row r="10" spans="1:2" ht="99.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="11" spans="1:2" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -1695,181 +1763,310 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:E10"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{85CFB8D1-FD16-4EF9-A991-1C12A9B050E6}">
+  <dimension ref="A1:E18"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="20" customWidth="1"/>
+    <col min="1" max="1" width="18" customWidth="1"/>
     <col min="2" max="2" width="22" customWidth="1"/>
     <col min="3" max="4" width="16" customWidth="1"/>
-    <col min="5" max="5" width="48" customWidth="1"/>
+    <col min="5" max="5" width="52" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="30" t="s">
+        <v>141</v>
+      </c>
+      <c r="B1" s="30"/>
+      <c r="C1" s="30"/>
+      <c r="D1" s="30"/>
+      <c r="E1" s="30"/>
+    </row>
+    <row r="2" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="31" t="s">
+        <v>140</v>
+      </c>
+      <c r="B2" s="31"/>
+      <c r="C2" s="31"/>
+      <c r="D2" s="31"/>
+      <c r="E2" s="31"/>
+    </row>
+    <row r="3" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="17" t="s">
+        <v>43</v>
+      </c>
+      <c r="B3" s="17" t="s">
+        <v>44</v>
+      </c>
+      <c r="C3" s="17" t="s">
+        <v>139</v>
+      </c>
+      <c r="D3" s="17" t="s">
+        <v>138</v>
+      </c>
+      <c r="E3" s="17" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="18" t="s">
+        <v>46</v>
+      </c>
+      <c r="B4" s="19" t="s">
+        <v>137</v>
+      </c>
+      <c r="C4" s="6" t="s">
+        <v>129</v>
+      </c>
+      <c r="D4" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="E4" s="19" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" ht="46.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="18" t="s">
+        <v>46</v>
+      </c>
+      <c r="B5" s="8" t="s">
+        <v>135</v>
+      </c>
+      <c r="C5" s="7" t="s">
+        <v>126</v>
+      </c>
+      <c r="D5" s="7" t="s">
+        <v>122</v>
+      </c>
+      <c r="E5" s="8" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" ht="34.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="18" t="s">
+        <v>46</v>
+      </c>
+      <c r="B6" s="19" t="s">
+        <v>133</v>
+      </c>
+      <c r="C6" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="D6" s="6" t="s">
+        <v>132</v>
+      </c>
+      <c r="E6" s="19" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" ht="46.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="20" t="s">
+        <v>46</v>
+      </c>
+      <c r="B7" s="8" t="s">
+        <v>130</v>
+      </c>
+      <c r="C7" s="7" t="s">
+        <v>129</v>
+      </c>
+      <c r="D7" s="7" t="s">
+        <v>126</v>
+      </c>
+      <c r="E7" s="8" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="20" t="s">
+        <v>46</v>
+      </c>
+      <c r="B8" s="19" t="s">
+        <v>127</v>
+      </c>
+      <c r="C8" s="6" t="s">
+        <v>126</v>
+      </c>
+      <c r="D8" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="E8" s="19" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="20" t="s">
+        <v>46</v>
+      </c>
+      <c r="B9" s="8" t="s">
+        <v>124</v>
+      </c>
+      <c r="C9" s="7" t="s">
+        <v>123</v>
+      </c>
+      <c r="D9" s="7" t="s">
+        <v>122</v>
+      </c>
+      <c r="E9" s="8" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="18" t="s">
+        <v>46</v>
+      </c>
+      <c r="B10" s="19" t="s">
+        <v>120</v>
+      </c>
+      <c r="C10" s="6" t="s">
+        <v>119</v>
+      </c>
+      <c r="D10" s="6" t="s">
+        <v>118</v>
+      </c>
+      <c r="E10" s="19" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="18" t="s">
+        <v>46</v>
+      </c>
+      <c r="B11" s="8" t="s">
+        <v>116</v>
+      </c>
+      <c r="C11" s="7" t="s">
+        <v>115</v>
+      </c>
+      <c r="D11" s="7" t="s">
+        <v>114</v>
+      </c>
+      <c r="E11" s="8" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" ht="48" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="20" t="s">
+        <v>46</v>
+      </c>
+      <c r="B12" s="19" t="s">
+        <v>112</v>
+      </c>
+      <c r="C12" s="6" t="s">
+        <v>104</v>
+      </c>
+      <c r="D12" s="6" t="s">
+        <v>101</v>
+      </c>
+      <c r="E12" s="19" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" ht="48.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="20" t="s">
+        <v>46</v>
+      </c>
+      <c r="B13" s="8" t="s">
+        <v>110</v>
+      </c>
+      <c r="C13" s="7" t="s">
+        <v>109</v>
+      </c>
+      <c r="D13" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="E13" s="8" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="21" t="s">
+        <v>107</v>
+      </c>
+      <c r="B14" s="19" t="s">
+        <v>106</v>
+      </c>
+      <c r="C14" s="6" t="s">
+        <v>105</v>
+      </c>
+      <c r="D14" s="6" t="s">
+        <v>104</v>
+      </c>
+      <c r="E14" s="19" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" ht="58.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="21" t="s">
+        <v>94</v>
+      </c>
+      <c r="B15" s="8" t="s">
+        <v>102</v>
+      </c>
+      <c r="C15" s="7" t="s">
+        <v>101</v>
+      </c>
+      <c r="D15" s="7" t="s">
+        <v>100</v>
+      </c>
+      <c r="E15" s="8" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" ht="59.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="21" t="s">
+        <v>94</v>
+      </c>
+      <c r="B16" s="19" t="s">
+        <v>98</v>
+      </c>
+      <c r="C16" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="D16" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="E16" s="19" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" ht="34.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="21" t="s">
+        <v>94</v>
+      </c>
+      <c r="B17" s="8" t="s">
+        <v>93</v>
+      </c>
+      <c r="C17" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="D17" s="7" t="s">
+        <v>91</v>
+      </c>
+      <c r="E17" s="8" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" ht="62.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="22" t="s">
+        <v>48</v>
+      </c>
+      <c r="B18" s="19" t="s">
         <v>89</v>
       </c>
-      <c r="B1" s="3"/>
-      <c r="C1" s="3"/>
-      <c r="D1" s="3"/>
-      <c r="E1" s="3"/>
-    </row>
-    <row r="2" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="23" t="s">
-        <v>43</v>
-      </c>
-      <c r="B2" s="23" t="s">
-        <v>44</v>
-      </c>
-      <c r="C2" s="23" t="s">
-        <v>45</v>
-      </c>
-      <c r="D2" s="23" t="s">
-        <v>46</v>
-      </c>
-      <c r="E2" s="23" t="s">
+      <c r="C18" s="6" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="3" spans="1:5" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="24" t="s">
-        <v>48</v>
-      </c>
-      <c r="B3" s="25" t="s">
-        <v>49</v>
-      </c>
-      <c r="C3" s="12" t="s">
-        <v>50</v>
-      </c>
-      <c r="D3" s="12" t="s">
-        <v>51</v>
-      </c>
-      <c r="E3" s="25" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="24" t="s">
-        <v>48</v>
-      </c>
-      <c r="B4" s="14" t="s">
-        <v>53</v>
-      </c>
-      <c r="C4" s="13" t="s">
-        <v>54</v>
-      </c>
-      <c r="D4" s="13" t="s">
-        <v>55</v>
-      </c>
-      <c r="E4" s="14" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="26" t="s">
-        <v>48</v>
-      </c>
-      <c r="B5" s="25" t="s">
-        <v>57</v>
-      </c>
-      <c r="C5" s="12" t="s">
-        <v>58</v>
-      </c>
-      <c r="D5" s="12" t="s">
-        <v>59</v>
-      </c>
-      <c r="E5" s="25" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="24" t="s">
-        <v>48</v>
-      </c>
-      <c r="B6" s="14" t="s">
-        <v>61</v>
-      </c>
-      <c r="C6" s="13" t="s">
-        <v>62</v>
-      </c>
-      <c r="D6" s="13" t="s">
-        <v>63</v>
-      </c>
-      <c r="E6" s="14" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="24" t="s">
-        <v>48</v>
-      </c>
-      <c r="B7" s="25" t="s">
-        <v>65</v>
-      </c>
-      <c r="C7" s="12" t="s">
-        <v>66</v>
-      </c>
-      <c r="D7" s="12" t="s">
-        <v>67</v>
-      </c>
-      <c r="E7" s="25" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="26" t="s">
-        <v>48</v>
-      </c>
-      <c r="B8" s="14" t="s">
-        <v>69</v>
-      </c>
-      <c r="C8" s="13" t="s">
-        <v>70</v>
-      </c>
-      <c r="D8" s="13" t="s">
-        <v>71</v>
-      </c>
-      <c r="E8" s="14" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="27" t="s">
-        <v>73</v>
-      </c>
-      <c r="B9" s="25" t="s">
-        <v>74</v>
-      </c>
-      <c r="C9" s="12" t="s">
-        <v>18</v>
-      </c>
-      <c r="D9" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="E9" s="25" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="28" t="s">
-        <v>77</v>
-      </c>
-      <c r="B10" s="14" t="s">
-        <v>78</v>
-      </c>
-      <c r="C10" s="13" t="s">
-        <v>18</v>
-      </c>
-      <c r="D10" s="13" t="s">
-        <v>79</v>
-      </c>
-      <c r="E10" s="14" t="s">
-        <v>80</v>
+      <c r="D18" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="E18" s="19" t="s">
+        <v>87</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="2">
     <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A2:E2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>